<commit_message>
test: update test credentials to match actual roles (COLLEGE_ADMIN, FACULTY_ADVISOR, STUDENT_ORGANIZER, VOLUNTEER, DEPARTMENT_APPROVER)
</commit_message>
<xml_diff>
--- a/test_data/test_credentials.xlsx
+++ b/test_data/test_credentials.xlsx
@@ -429,13 +429,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
@@ -496,12 +496,12 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Event Organizer</t>
+          <t>Faculty Advisor</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>organizer@college.edu</t>
+          <t>faculty.advisor@college.edu</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -511,24 +511,24 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>ORGANIZER</t>
+          <t>FACULTY_ADVISOR</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Organizer@123</t>
+          <t>FacultyAdvisor@123</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Event Approver</t>
+          <t>Student Organizer</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>approver@college.edu</t>
+          <t>organizer@college.edu</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
@@ -538,24 +538,24 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>APPROVER</t>
+          <t>STUDENT_ORGANIZER</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Approver@123</t>
+          <t>StudentOrganizer@123</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Regular User</t>
+          <t>Event Volunteer</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>user@college.edu</t>
+          <t>volunteer@college.edu</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -565,12 +565,39 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>USER</t>
+          <t>VOLUNTEER</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>User@123</t>
+          <t>Volunteer@123</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Department Approver</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>approver@college.edu</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>college.edu</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>DEPARTMENT_APPROVER</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>DeptApprover@123</t>
         </is>
       </c>
     </row>

</xml_diff>